<commit_message>
Add step-by-step explanations, paste grid and ID-based hierarchy
- Ícone i em cada análise com resumo no tooltip; ao clicar, painel móvel
  com o passo a passo calculado sobre os dados carregados, com seletores
  de exemplo (coorte, grupo, KPI, cliente) e glossário em tooltips.
- Colar abre um modal em tabela com as colunas do modelo (cores por
  obrigatoriedade), reconhece cabeçalho, permite remapear colunas e
  importa. Ver reabre o modal com os dados já carregados.
- Hierarquia por id_group, id_org, id_product e hierarchy_type; linhas
  de grupo/organização com filhos só nomeiam a hierarquia.
- Consulta de perfil de qualidade dos dados (sql/perfil_dados.sql).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modelos/modelo_churn.xlsx
+++ b/modelos/modelo_churn.xlsx
@@ -193,95 +193,115 @@
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>importante: Hierarquia: grupo econômico.</t>
+        <t>importante: O que a linha representa: grupo, organizacao ou produto. Linhas de grupo ou organização com linhas abaixo só dão nome à hierarquia.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>importante: Hierarquia: organização (o próprio cliente). Pode ser name_contract no lugar.</t>
+        <t>importante: Hierarquia: ID do grupo econômico.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>importante: Hierarquia: produto contratado, quando o cliente tem uma linha por produto.</t>
+        <t>importante: Hierarquia: nome do grupo econômico.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
+        <t>importante: Hierarquia: ID da organização (o próprio cliente).</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>importante: Hierarquia: ID do produto contratado, quando o cliente tem uma linha por produto.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>importante: Hierarquia: nome do produto.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
         <t>importante: Perfil: setor.</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="L1" authorId="0" shapeId="0">
       <text>
         <t>importante: Perfil: porte.</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <t>importante: Perfil: UF.</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
+    <comment ref="N1" authorId="0" shapeId="0">
       <text>
         <t>importante: Perfil: etapa do ciclo de vida.</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
+    <comment ref="O1" authorId="0" shapeId="0">
       <text>
         <t>importante: Perfil: nome do CSM responsável (texto, como os demais campos de perfil).</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <t>importante: Motivo do cancelamento (tag).</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="Q1" authorId="0" shapeId="0">
       <text>
         <t>importante: Descrição do motivo.</t>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
+    <comment ref="R1" authorId="0" shapeId="0">
       <text>
         <t>importante: Receita mensal da linha. Ex.: custom_fields-&gt;&gt;'mrr'.</t>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <t>opcional: CNPJ da organização.</t>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
       <text>
         <t>opcional: ID no sistema anterior.</t>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
+    <comment ref="U1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Nome do contrato.</t>
       </text>
     </comment>
-    <comment ref="R1" authorId="0" shapeId="0">
+    <comment ref="V1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Cidade.</t>
       </text>
     </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
+    <comment ref="W1" authorId="0" shapeId="0">
       <text>
         <t>opcional: País.</t>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
+    <comment ref="X1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Responsável de suporte. Vira perfil se tiver poucos valores.</t>
       </text>
     </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
+    <comment ref="Y1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Vendedor. Vira perfil se tiver poucos valores.</t>
       </text>
     </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
+    <comment ref="Z1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Responsável pelo onboarding. Vira perfil se tiver poucos valores.</t>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
+    <comment ref="AA1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Data da etapa atual.</t>
       </text>
@@ -654,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -850,7 +870,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>group</t>
+          <t>hierarchy_type</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -860,7 +880,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Hierarquia: grupo econômico.</t>
+          <t>O que a linha representa: grupo, organizacao ou produto. Linhas de grupo ou organização com linhas abaixo só dão nome à hierarquia.</t>
         </is>
       </c>
     </row>
@@ -872,7 +892,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>cnpj</t>
+          <t>id_group</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -882,7 +902,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Hierarquia: organização (o próprio cliente). Pode ser name_contract no lugar.</t>
+          <t>Hierarquia: ID do grupo econômico.</t>
         </is>
       </c>
     </row>
@@ -894,7 +914,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>product</t>
+          <t>group</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -904,7 +924,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Hierarquia: produto contratado, quando o cliente tem uma linha por produto.</t>
+          <t>Hierarquia: nome do grupo econômico.</t>
         </is>
       </c>
     </row>
@@ -916,7 +936,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>industry</t>
+          <t>id_org</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -926,7 +946,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Perfil: setor.</t>
+          <t>Hierarquia: ID da organização (o próprio cliente).</t>
         </is>
       </c>
     </row>
@@ -938,7 +958,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>size</t>
+          <t>id_product</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -948,7 +968,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Perfil: porte.</t>
+          <t>Hierarquia: ID do produto contratado, quando o cliente tem uma linha por produto.</t>
         </is>
       </c>
     </row>
@@ -960,7 +980,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>product</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -970,7 +990,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Perfil: UF.</t>
+          <t>Hierarquia: nome do produto.</t>
         </is>
       </c>
     </row>
@@ -982,7 +1002,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>stage</t>
+          <t>industry</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -992,7 +1012,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Perfil: etapa do ciclo de vida.</t>
+          <t>Perfil: setor.</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1024,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>cs_owner</t>
+          <t>size</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1014,7 +1034,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Perfil: nome do CSM responsável (texto, como os demais campos de perfil).</t>
+          <t>Perfil: porte.</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1046,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>cancel_tag</t>
+          <t>state</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -1036,7 +1056,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Motivo do cancelamento (tag).</t>
+          <t>Perfil: UF.</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1068,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>cancel_description</t>
+          <t>stage</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1058,7 +1078,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Descrição do motivo.</t>
+          <t>Perfil: etapa do ciclo de vida.</t>
         </is>
       </c>
     </row>
@@ -1070,7 +1090,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>mrr</t>
+          <t>cs_owner</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -1080,7 +1100,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Receita mensal da linha. Ex.: custom_fields-&gt;&gt;'mrr'.</t>
+          <t>Perfil: nome do CSM responsável (texto, como os demais campos de perfil).</t>
         </is>
       </c>
     </row>
@@ -1092,17 +1112,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>id_legacy</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>opcional</t>
+          <t>cancel_tag</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>ID no sistema anterior.</t>
+          <t>Motivo do cancelamento (tag).</t>
         </is>
       </c>
     </row>
@@ -1114,17 +1134,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>name_contract</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>opcional</t>
+          <t>cancel_description</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Nome do contrato.</t>
+          <t>Descrição do motivo.</t>
         </is>
       </c>
     </row>
@@ -1136,17 +1156,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>city</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>opcional</t>
+          <t>mrr</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Cidade.</t>
+          <t>Receita mensal da linha. Ex.: custom_fields-&gt;&gt;'mrr'.</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1178,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>country</t>
+          <t>cnpj</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1168,7 +1188,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>País.</t>
+          <t>CNPJ da organização.</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1200,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>support_owner</t>
+          <t>id_legacy</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1190,7 +1210,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Responsável de suporte. Vira perfil se tiver poucos valores.</t>
+          <t>ID no sistema anterior.</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1222,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>sales_owner</t>
+          <t>name_contract</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1212,7 +1232,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Vendedor. Vira perfil se tiver poucos valores.</t>
+          <t>Nome do contrato.</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1244,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>onboarding_owner</t>
+          <t>city</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1234,7 +1254,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Responsável pelo onboarding. Vira perfil se tiver poucos valores.</t>
+          <t>Cidade.</t>
         </is>
       </c>
     </row>
@@ -1246,7 +1266,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>dt_stage</t>
+          <t>country</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1256,95 +1276,95 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Data da etapa atual.</t>
+          <t>País.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>kpi</t>
+          <t>customer</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>id_customer</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>obrigatório</t>
+          <t>support_owner</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>opcional</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>ID da linha de cliente (customer.id).</t>
+          <t>Responsável de suporte. Vira perfil se tiver poucos valores.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>kpi</t>
+          <t>customer</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>type</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>obrigatório</t>
+          <t>sales_owner</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>opcional</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>ID do tipo de KPI (kpi_type.id).</t>
+          <t>Vendedor. Vira perfil se tiver poucos valores.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>kpi</t>
+          <t>customer</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>obrigatório</t>
+          <t>onboarding_owner</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>opcional</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Valor do KPI.</t>
+          <t>Responsável pelo onboarding. Vira perfil se tiver poucos valores.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>kpi</t>
+          <t>customer</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ref_date</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>importante</t>
+          <t>dt_stage</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>opcional</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Data da leitura. Sem ela, vale a média das linhas do cliente.</t>
+          <t>Data da etapa atual.</t>
         </is>
       </c>
     </row>
@@ -1356,17 +1376,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>kpi_name</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>importante</t>
+          <t>id_customer</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Nome do KPI (kpi_type.name). Sem ele, aparece como KPI 1, KPI 2…</t>
+          <t>ID da linha de cliente (customer.id).</t>
         </is>
       </c>
     </row>
@@ -1378,17 +1398,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>inv_proportional</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>importante</t>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>kpi_type.inv_proportional. true = valor maior é pior.</t>
+          <t>ID do tipo de KPI (kpi_type.id).</t>
         </is>
       </c>
     </row>
@@ -1400,73 +1420,73 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>opcional</t>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Unidade (kpi_type.unit).</t>
+          <t>Valor do KPI.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>cancelamentos</t>
+          <t>kpi</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>id_customer</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>obrigatório</t>
+          <t>ref_date</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>ID da linha de cliente. Só use se o cancelamento não estiver em customer.</t>
+          <t>Data da leitura. Sem ela, vale a média das linhas do cliente.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>cancelamentos</t>
+          <t>kpi</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>dt_cancel</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>obrigatório</t>
+          <t>kpi_name</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Data do cancelamento.</t>
+          <t>Nome do KPI (kpi_type.name). Sem ele, aparece como KPI 1, KPI 2…</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>cancelamentos</t>
+          <t>kpi</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>cancel_tag</t>
+          <t>inv_proportional</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -1476,27 +1496,115 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Motivo do cancelamento.</t>
+          <t>kpi_type.inv_proportional. true = valor maior é pior.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>kpi</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>opcional</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Unidade (kpi_type.unit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>cancelamentos</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>id_customer</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ID da linha de cliente. Só use se o cancelamento não estiver em customer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>cancelamentos</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>dt_cancel</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Data do cancelamento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>cancelamentos</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>cancel_tag</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Motivo do cancelamento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>cancelamentos</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
         <is>
           <t>mrr_perdido</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>opcional</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>MRR perdido, se diferente do mrr em customer.</t>
         </is>
@@ -1513,14 +1621,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:AA1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
@@ -1529,16 +1637,20 @@
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="17" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="17" customWidth="1" min="20" max="20"/>
-    <col width="15" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="17" customWidth="1" min="24" max="24"/>
+    <col width="15" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1564,95 +1676,115 @@
       </c>
       <c r="E1" s="6" t="inlineStr">
         <is>
+          <t>hierarchy_type</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>id_group</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
           <t>group</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>id_org</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>id_product</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>industry</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="N1" s="6" t="inlineStr">
+        <is>
+          <t>stage</t>
+        </is>
+      </c>
+      <c r="O1" s="6" t="inlineStr">
+        <is>
+          <t>cs_owner</t>
+        </is>
+      </c>
+      <c r="P1" s="6" t="inlineStr">
+        <is>
+          <t>cancel_tag</t>
+        </is>
+      </c>
+      <c r="Q1" s="6" t="inlineStr">
+        <is>
+          <t>cancel_description</t>
+        </is>
+      </c>
+      <c r="R1" s="6" t="inlineStr">
+        <is>
+          <t>mrr</t>
+        </is>
+      </c>
+      <c r="S1" s="7" t="inlineStr">
         <is>
           <t>cnpj</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="H1" s="6" t="inlineStr">
-        <is>
-          <t>industry</t>
-        </is>
-      </c>
-      <c r="I1" s="6" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" s="6" t="inlineStr">
-        <is>
-          <t>state</t>
-        </is>
-      </c>
-      <c r="K1" s="6" t="inlineStr">
-        <is>
-          <t>stage</t>
-        </is>
-      </c>
-      <c r="L1" s="6" t="inlineStr">
-        <is>
-          <t>cs_owner</t>
-        </is>
-      </c>
-      <c r="M1" s="6" t="inlineStr">
-        <is>
-          <t>cancel_tag</t>
-        </is>
-      </c>
-      <c r="N1" s="6" t="inlineStr">
-        <is>
-          <t>cancel_description</t>
-        </is>
-      </c>
-      <c r="O1" s="6" t="inlineStr">
-        <is>
-          <t>mrr</t>
-        </is>
-      </c>
-      <c r="P1" s="7" t="inlineStr">
+      <c r="T1" s="7" t="inlineStr">
         <is>
           <t>id_legacy</t>
         </is>
       </c>
-      <c r="Q1" s="7" t="inlineStr">
+      <c r="U1" s="7" t="inlineStr">
         <is>
           <t>name_contract</t>
         </is>
       </c>
-      <c r="R1" s="7" t="inlineStr">
+      <c r="V1" s="7" t="inlineStr">
         <is>
           <t>city</t>
         </is>
       </c>
-      <c r="S1" s="7" t="inlineStr">
+      <c r="W1" s="7" t="inlineStr">
         <is>
           <t>country</t>
         </is>
       </c>
-      <c r="T1" s="7" t="inlineStr">
+      <c r="X1" s="7" t="inlineStr">
         <is>
           <t>support_owner</t>
         </is>
       </c>
-      <c r="U1" s="7" t="inlineStr">
+      <c r="Y1" s="7" t="inlineStr">
         <is>
           <t>sales_owner</t>
         </is>
       </c>
-      <c r="V1" s="7" t="inlineStr">
+      <c r="Z1" s="7" t="inlineStr">
         <is>
           <t>onboarding_owner</t>
         </is>
       </c>
-      <c r="W1" s="7" t="inlineStr">
+      <c r="AA1" s="7" t="inlineStr">
         <is>
           <t>dt_stage</t>
         </is>

</xml_diff>

<commit_message>
Ficha do cliente, quadro de risco, relatório exportável, adoção por perfil e NRR
- Ficha lateral do cliente: pontos de cada KPI no score, KPIs mês a mês, linhas, motivo e nota
- Quadro de risco (A abordar, Em contato, Plano de ação, Resolvido) com arrastar,
  seletor por teclado e cartão vermelho após 7 dias; fica no navegador
- Exportar relatório: .zip com painel de diagnóstico embutido, análises em CSV
  (vírgula decimal, UTF-8) e os dados de entrada
- Tour por papel (CSM termina na Carteira, Head de CS na Visão geral) trocando de área
- Dicas pontuais uma por vez e painel de uso local
- Teste no tempo aprende pesos só com dados até a data T; NRR por mrr_12m_atras
  (SenseData calcula pelos contratos vigentes há 12 meses)
- Roadmap com decisões tomadas e status de entrega; README e testes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modelos/modelo_churn.xlsx
+++ b/modelos/modelo_churn.xlsx
@@ -263,45 +263,50 @@
     </comment>
     <comment ref="S1" authorId="0" shapeId="0">
       <text>
+        <t>opcional: MRR da linha 12 meses antes. Com ele o relatório calcula o NRR.</t>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
         <t>opcional: CNPJ da organização.</t>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
+    <comment ref="U1" authorId="0" shapeId="0">
       <text>
         <t>opcional: ID no sistema anterior.</t>
       </text>
     </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
+    <comment ref="V1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Nome do contrato.</t>
       </text>
     </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
+    <comment ref="W1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Cidade.</t>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
+    <comment ref="X1" authorId="0" shapeId="0">
       <text>
         <t>opcional: País.</t>
       </text>
     </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
+    <comment ref="Y1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Responsável de suporte. Vira perfil se tiver poucos valores.</t>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
+    <comment ref="Z1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Vendedor. Vira perfil se tiver poucos valores.</t>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
+    <comment ref="AA1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Responsável pelo onboarding. Vira perfil se tiver poucos valores.</t>
       </text>
     </comment>
-    <comment ref="AA1" authorId="0" shapeId="0">
+    <comment ref="AB1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Data da etapa atual.</t>
       </text>
@@ -674,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1178,7 +1183,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>cnpj</t>
+          <t>mrr_12m_atras</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1188,7 +1193,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>CNPJ da organização.</t>
+          <t>MRR da linha 12 meses antes. Com ele o relatório calcula o NRR.</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1205,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>id_legacy</t>
+          <t>cnpj</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1210,7 +1215,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>ID no sistema anterior.</t>
+          <t>CNPJ da organização.</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1227,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>name_contract</t>
+          <t>id_legacy</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1232,7 +1237,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Nome do contrato.</t>
+          <t>ID no sistema anterior.</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1249,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>name_contract</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1254,7 +1259,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Cidade.</t>
+          <t>Nome do contrato.</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1271,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>country</t>
+          <t>city</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1276,7 +1281,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>País.</t>
+          <t>Cidade.</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1293,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>support_owner</t>
+          <t>country</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1298,7 +1303,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Responsável de suporte. Vira perfil se tiver poucos valores.</t>
+          <t>País.</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1315,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>sales_owner</t>
+          <t>support_owner</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1320,7 +1325,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Vendedor. Vira perfil se tiver poucos valores.</t>
+          <t>Responsável de suporte. Vira perfil se tiver poucos valores.</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1337,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>onboarding_owner</t>
+          <t>sales_owner</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1342,7 +1347,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Responsável pelo onboarding. Vira perfil se tiver poucos valores.</t>
+          <t>Vendedor. Vira perfil se tiver poucos valores.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1359,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>dt_stage</t>
+          <t>onboarding_owner</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1364,29 +1369,29 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Data da etapa atual.</t>
+          <t>Responsável pelo onboarding. Vira perfil se tiver poucos valores.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>kpi</t>
+          <t>customer</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>id_customer</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>obrigatório</t>
+          <t>dt_stage</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>opcional</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>ID da linha de cliente (customer.id).</t>
+          <t>Data da etapa atual.</t>
         </is>
       </c>
     </row>
@@ -1398,7 +1403,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>id_customer</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -1408,7 +1413,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>ID do tipo de KPI (kpi_type.id).</t>
+          <t>ID da linha de cliente (customer.id).</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1425,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>type</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -1430,7 +1435,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Valor do KPI.</t>
+          <t>ID do tipo de KPI (kpi_type.id).</t>
         </is>
       </c>
     </row>
@@ -1442,17 +1447,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ref_date</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>importante</t>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Data da leitura. Sem ela, vale a média das linhas do cliente.</t>
+          <t>Valor do KPI.</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1469,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>kpi_name</t>
+          <t>ref_date</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -1474,7 +1479,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Nome do KPI (kpi_type.name). Sem ele, aparece como KPI 1, KPI 2…</t>
+          <t>Data da leitura. Sem ela, vale a média das linhas do cliente.</t>
         </is>
       </c>
     </row>
@@ -1486,7 +1491,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>inv_proportional</t>
+          <t>kpi_name</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -1496,7 +1501,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>kpi_type.inv_proportional. true = valor maior é pior.</t>
+          <t>Nome do KPI (kpi_type.name). Sem ele, aparece como KPI 1, KPI 2…</t>
         </is>
       </c>
     </row>
@@ -1508,39 +1513,39 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>opcional</t>
+          <t>inv_proportional</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Unidade (kpi_type.unit).</t>
+          <t>kpi_type.inv_proportional. true = valor maior é pior.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>cancelamentos</t>
+          <t>kpi</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>id_customer</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>obrigatório</t>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>opcional</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>ID da linha de cliente. Só use se o cancelamento não estiver em customer.</t>
+          <t>Unidade (kpi_type.unit).</t>
         </is>
       </c>
     </row>
@@ -1552,7 +1557,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>dt_cancel</t>
+          <t>id_customer</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -1562,7 +1567,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Data do cancelamento.</t>
+          <t>ID da linha de cliente. Só use se o cancelamento não estiver em customer.</t>
         </is>
       </c>
     </row>
@@ -1574,17 +1579,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>cancel_tag</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>importante</t>
+          <t>dt_cancel</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Motivo do cancelamento.</t>
+          <t>Data do cancelamento.</t>
         </is>
       </c>
     </row>
@@ -1596,15 +1601,37 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
+          <t>cancel_tag</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Motivo do cancelamento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>cancelamentos</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
           <t>mrr_perdido</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>opcional</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>MRR perdido, se diferente do mrr em customer.</t>
         </is>
@@ -1621,7 +1648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1642,15 +1669,16 @@
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="22" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="17" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="17" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="17" customWidth="1" min="24" max="24"/>
-    <col width="15" customWidth="1" min="25" max="25"/>
-    <col width="20" customWidth="1" min="26" max="26"/>
-    <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="17" customWidth="1" min="25" max="25"/>
+    <col width="15" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1746,45 +1774,50 @@
       </c>
       <c r="S1" s="7" t="inlineStr">
         <is>
+          <t>mrr_12m_atras</t>
+        </is>
+      </c>
+      <c r="T1" s="7" t="inlineStr">
+        <is>
           <t>cnpj</t>
         </is>
       </c>
-      <c r="T1" s="7" t="inlineStr">
+      <c r="U1" s="7" t="inlineStr">
         <is>
           <t>id_legacy</t>
         </is>
       </c>
-      <c r="U1" s="7" t="inlineStr">
+      <c r="V1" s="7" t="inlineStr">
         <is>
           <t>name_contract</t>
         </is>
       </c>
-      <c r="V1" s="7" t="inlineStr">
+      <c r="W1" s="7" t="inlineStr">
         <is>
           <t>city</t>
         </is>
       </c>
-      <c r="W1" s="7" t="inlineStr">
+      <c r="X1" s="7" t="inlineStr">
         <is>
           <t>country</t>
         </is>
       </c>
-      <c r="X1" s="7" t="inlineStr">
+      <c r="Y1" s="7" t="inlineStr">
         <is>
           <t>support_owner</t>
         </is>
       </c>
-      <c r="Y1" s="7" t="inlineStr">
+      <c r="Z1" s="7" t="inlineStr">
         <is>
           <t>sales_owner</t>
         </is>
       </c>
-      <c r="Z1" s="7" t="inlineStr">
+      <c r="AA1" s="7" t="inlineStr">
         <is>
           <t>onboarding_owner</t>
         </is>
       </c>
-      <c r="AA1" s="7" t="inlineStr">
+      <c r="AB1" s="7" t="inlineStr">
         <is>
           <t>dt_stage</t>
         </is>

</xml_diff>

<commit_message>
Sinais de churn e assinatura de cada motivo de cancelamento
- Fontes opcionais Tickets, NPS, Tarefas e interações e Uso (colunas da API v2) e sponsor_desde em Clientes
- Importação SenseData de support_tickets, nps, tasks, tasks_checkin, customers_notes,
  usage_time, default_usage e contacts (sponsor), últimos 18 meses; fonte sem acesso é pulada
- Fotos mensais com variáveis calculadas só até cada data; pedidos de cancelamento e
  tarefas de retenção ficam fora
- Diagnóstico: matriz motivo x família de sinais e detalhe com efeito, antecedência e estabilidade
- Ficha do cliente: 'Parecido com quem saiu por X'; exportação com assinaturas e fotos mensais
- Exemplo com sinais por motivo (gerador separado, números atuais preservados), API simulada,
  modelos de planilha, tools/gerar_exemplos.mjs e testes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modelos/modelo_churn.xlsx
+++ b/modelos/modelo_churn.xlsx
@@ -11,6 +11,10 @@
     <sheet name="customer" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="kpi" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="cancelamentos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="tickets" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="nps" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="tarefas" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="uso" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -268,45 +272,50 @@
     </comment>
     <comment ref="T1" authorId="0" shapeId="0">
       <text>
+        <t>opcional: Desde quando o sponsor atual é o sponsor (data de cadastro do contato).</t>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0">
+      <text>
         <t>opcional: CNPJ da organização.</t>
       </text>
     </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
+    <comment ref="V1" authorId="0" shapeId="0">
       <text>
         <t>opcional: ID no sistema anterior.</t>
       </text>
     </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
+    <comment ref="W1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Nome do contrato.</t>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
+    <comment ref="X1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Cidade.</t>
       </text>
     </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
+    <comment ref="Y1" authorId="0" shapeId="0">
       <text>
         <t>opcional: País.</t>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
+    <comment ref="Z1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Responsável de suporte. Vira perfil se tiver poucos valores.</t>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
+    <comment ref="AA1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Vendedor. Vira perfil se tiver poucos valores.</t>
       </text>
     </comment>
-    <comment ref="AA1" authorId="0" shapeId="0">
+    <comment ref="AB1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Responsável pelo onboarding. Vira perfil se tiver poucos valores.</t>
       </text>
     </comment>
-    <comment ref="AB1" authorId="0" shapeId="0">
+    <comment ref="AC1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Data da etapa atual.</t>
       </text>
@@ -384,6 +393,181 @@
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <t>opcional: MRR perdido, se diferente do mrr em customer.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>modelo</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>obrigatório: ID da linha de cliente.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>obrigatório: Data de abertura do ticket.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>importante: Data de resolução. Vazio = aberto.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>importante: Prazo (SLA).</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>importante: Prioridade. Alta e urgente contam como graves.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>importante: Categoria.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>opcional: Tipo.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>opcional: Título. Usado só para tirar pedidos de cancelamento.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>modelo</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>obrigatório: ID da linha de cliente.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>obrigatório: Data da resposta.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>obrigatório: Nota de 0 a 10.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>importante: Cargo de quem respondeu. Sponsor, decisor ou diretor contam como sponsor.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>opcional: Tags da resposta.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>modelo</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>obrigatório: ID da linha de cliente.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>importante: tarefa, visita ou nota.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>importante: Tipo da tarefa. Reunião, call, QBR ou visita contam como reunião.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>obrigatório: Data de criação.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>importante: Prazo.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>importante: Data de conclusão.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>opcional: Nome do playbook que gerou a tarefa.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>opcional: Tags.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>modelo</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>obrigatório: ID da linha de cliente.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>obrigatório: Mês de referência.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>obrigatório: Usuários ativos no mês.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>importante: Usuários contratados.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>opcional: Tempo de uso no mês.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>opcional: Quantos módulos foram usados no mês.</t>
       </text>
     </comment>
   </commentList>
@@ -679,7 +863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1205,7 +1389,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>cnpj</t>
+          <t>sponsor_desde</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1215,7 +1399,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CNPJ da organização.</t>
+          <t>Desde quando o sponsor atual é o sponsor (data de cadastro do contato).</t>
         </is>
       </c>
     </row>
@@ -1227,7 +1411,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>id_legacy</t>
+          <t>cnpj</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1237,7 +1421,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>ID no sistema anterior.</t>
+          <t>CNPJ da organização.</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1433,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>name_contract</t>
+          <t>id_legacy</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1259,7 +1443,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Nome do contrato.</t>
+          <t>ID no sistema anterior.</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1455,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>name_contract</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1281,7 +1465,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Cidade.</t>
+          <t>Nome do contrato.</t>
         </is>
       </c>
     </row>
@@ -1293,7 +1477,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>country</t>
+          <t>city</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1303,7 +1487,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>País.</t>
+          <t>Cidade.</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1499,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>support_owner</t>
+          <t>country</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1325,7 +1509,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Responsável de suporte. Vira perfil se tiver poucos valores.</t>
+          <t>País.</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1521,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>sales_owner</t>
+          <t>support_owner</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1347,7 +1531,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Vendedor. Vira perfil se tiver poucos valores.</t>
+          <t>Responsável de suporte. Vira perfil se tiver poucos valores.</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1543,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>onboarding_owner</t>
+          <t>sales_owner</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1369,7 +1553,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Responsável pelo onboarding. Vira perfil se tiver poucos valores.</t>
+          <t>Vendedor. Vira perfil se tiver poucos valores.</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1565,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>dt_stage</t>
+          <t>onboarding_owner</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1391,29 +1575,29 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Data da etapa atual.</t>
+          <t>Responsável pelo onboarding. Vira perfil se tiver poucos valores.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>kpi</t>
+          <t>customer</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>id_customer</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>obrigatório</t>
+          <t>dt_stage</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>opcional</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>ID da linha de cliente (customer.id).</t>
+          <t>Data da etapa atual.</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1609,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>id_customer</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -1435,7 +1619,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>ID do tipo de KPI (kpi_type.id).</t>
+          <t>ID da linha de cliente (customer.id).</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1631,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>type</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -1457,7 +1641,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Valor do KPI.</t>
+          <t>ID do tipo de KPI (kpi_type.id).</t>
         </is>
       </c>
     </row>
@@ -1469,17 +1653,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ref_date</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>importante</t>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Data da leitura. Sem ela, vale a média das linhas do cliente.</t>
+          <t>Valor do KPI.</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1675,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>kpi_name</t>
+          <t>ref_date</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -1501,7 +1685,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Nome do KPI (kpi_type.name). Sem ele, aparece como KPI 1, KPI 2…</t>
+          <t>Data da leitura. Sem ela, vale a média das linhas do cliente.</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1697,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>inv_proportional</t>
+          <t>kpi_name</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -1523,7 +1707,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>kpi_type.inv_proportional. true = valor maior é pior.</t>
+          <t>Nome do KPI (kpi_type.name). Sem ele, aparece como KPI 1, KPI 2…</t>
         </is>
       </c>
     </row>
@@ -1535,39 +1719,39 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>opcional</t>
+          <t>inv_proportional</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Unidade (kpi_type.unit).</t>
+          <t>kpi_type.inv_proportional. true = valor maior é pior.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>cancelamentos</t>
+          <t>kpi</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>id_customer</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>obrigatório</t>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>opcional</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>ID da linha de cliente. Só use se o cancelamento não estiver em customer.</t>
+          <t>Unidade (kpi_type.unit).</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1763,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>dt_cancel</t>
+          <t>id_customer</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -1589,7 +1773,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Data do cancelamento.</t>
+          <t>ID da linha de cliente. Só use se o cancelamento não estiver em customer.</t>
         </is>
       </c>
     </row>
@@ -1601,17 +1785,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>cancel_tag</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>importante</t>
+          <t>dt_cancel</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Motivo do cancelamento.</t>
+          <t>Data do cancelamento.</t>
         </is>
       </c>
     </row>
@@ -1623,17 +1807,633 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>cancel_tag</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Motivo do cancelamento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>cancelamentos</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
           <t>mrr_perdido</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>opcional</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>MRR perdido, se diferente do mrr em customer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>tickets</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>id_customer</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ID da linha de cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>tickets</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>created_on</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Data de abertura do ticket.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>tickets</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Data de resolução. Vazio = aberto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>tickets</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>expire_date</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Prazo (SLA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>tickets</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Prioridade. Alta e urgente contam como graves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>tickets</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Categoria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>tickets</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>opcional</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Tipo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>tickets</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>opcional</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Título. Usado só para tirar pedidos de cancelamento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>id_customer</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>ID da linha de cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>survey_date</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Data da resposta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Nota de 0 a 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Cargo de quem respondeu. Sponsor, decisor ou diretor contam como sponsor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>tags</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>opcional</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Tags da resposta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>tarefas</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>id_customer</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>ID da linha de cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>tarefas</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>tarefa, visita ou nota.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>tarefas</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Tipo da tarefa. Reunião, call, QBR ou visita contam como reunião.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>tarefas</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>created_on</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Data de criação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>tarefas</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>due_date</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Prazo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>tarefas</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Data de conclusão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>tarefas</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>playbook</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>opcional</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Nome do playbook que gerou a tarefa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>tarefas</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>tags</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>opcional</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Tags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>uso</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>id_customer</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>ID da linha de cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>uso</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ref_date</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Mês de referência.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>uso</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>active_users</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Usuários ativos no mês.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>uso</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>contracted_users</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Usuários contratados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>uso</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>usage_time</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>opcional</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Tempo de uso no mês.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>uso</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>modules</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>opcional</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Quantos módulos foram usados no mês.</t>
         </is>
       </c>
     </row>
@@ -1648,7 +2448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AC1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1670,15 +2470,16 @@
     <col width="22" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
     <col width="17" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="17" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="17" customWidth="1" min="23" max="23"/>
     <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="17" customWidth="1" min="25" max="25"/>
-    <col width="15" customWidth="1" min="26" max="26"/>
-    <col width="20" customWidth="1" min="27" max="27"/>
-    <col width="14" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="17" customWidth="1" min="26" max="26"/>
+    <col width="15" customWidth="1" min="27" max="27"/>
+    <col width="20" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1779,45 +2580,50 @@
       </c>
       <c r="T1" s="7" t="inlineStr">
         <is>
+          <t>sponsor_desde</t>
+        </is>
+      </c>
+      <c r="U1" s="7" t="inlineStr">
+        <is>
           <t>cnpj</t>
         </is>
       </c>
-      <c r="U1" s="7" t="inlineStr">
+      <c r="V1" s="7" t="inlineStr">
         <is>
           <t>id_legacy</t>
         </is>
       </c>
-      <c r="V1" s="7" t="inlineStr">
+      <c r="W1" s="7" t="inlineStr">
         <is>
           <t>name_contract</t>
         </is>
       </c>
-      <c r="W1" s="7" t="inlineStr">
+      <c r="X1" s="7" t="inlineStr">
         <is>
           <t>city</t>
         </is>
       </c>
-      <c r="X1" s="7" t="inlineStr">
+      <c r="Y1" s="7" t="inlineStr">
         <is>
           <t>country</t>
         </is>
       </c>
-      <c r="Y1" s="7" t="inlineStr">
+      <c r="Z1" s="7" t="inlineStr">
         <is>
           <t>support_owner</t>
         </is>
       </c>
-      <c r="Z1" s="7" t="inlineStr">
+      <c r="AA1" s="7" t="inlineStr">
         <is>
           <t>sales_owner</t>
         </is>
       </c>
-      <c r="AA1" s="7" t="inlineStr">
+      <c r="AB1" s="7" t="inlineStr">
         <is>
           <t>onboarding_owner</t>
         </is>
       </c>
-      <c r="AB1" s="7" t="inlineStr">
+      <c r="AC1" s="7" t="inlineStr">
         <is>
           <t>dt_stage</t>
         </is>
@@ -1931,4 +2737,242 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>id_customer</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>created_on</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>expire_date</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>id_customer</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>survey_date</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>tags</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>id_customer</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>created_on</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>due_date</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>playbook</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>tags</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>id_customer</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>ref_date</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>active_users</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>contracted_users</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>usage_time</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>modules</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Contratos como sinal e casos para entrevista com os CSMs
- Fonte Contratos (start_date, end_date, monthly_payment, cycle) e importação de /v2/contracts com os sinais
- Variáveis: variação do valor contratado e redução em 90 dias, contratos encerrados e dias até a renovação
  pelo aniversário do início; o fim de um contrato ainda vigente nunca é lido (evita vazar a saída)
- Casos para entrevista por motivo (antecipado e não antecipado, com CSM), roteiro de 30 min e CSV
- docs/roteiro-entrevistas.md: plano, roteiro, registro e síntese
- Exemplo, API simulada, modelos de planilha e testes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modelos/modelo_churn.xlsx
+++ b/modelos/modelo_churn.xlsx
@@ -15,6 +15,7 @@
     <sheet name="nps" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="tarefas" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="uso" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="contratos" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -568,6 +569,41 @@
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <t>opcional: Quantos módulos foram usados no mês.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>modelo</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>obrigatório: ID da linha de cliente.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>obrigatório: Início da vigência.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>importante: Fim da vigência. Vazio = vigente.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>obrigatório: Valor mensal do contrato.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>importante: Ciclo de renovação em meses (12, anual, semestral...). Sem ele, conta 12.</t>
       </text>
     </comment>
   </commentList>
@@ -863,7 +899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D78"/>
+  <dimension ref="A1:D83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2434,6 +2470,116 @@
       <c r="D78" t="inlineStr">
         <is>
           <t>Quantos módulos foram usados no mês.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>contratos</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>id_customer</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>ID da linha de cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>contratos</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>start_date</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Início da vigência.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>contratos</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Fim da vigência. Vazio = vigente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>contratos</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>monthly_payment</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>obrigatório</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Valor mensal do contrato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>contratos</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>cycle</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>importante</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Ciclo de renovação em meses (12, anual, semestral...). Sem ele, conta 12.</t>
         </is>
       </c>
     </row>
@@ -2975,4 +3121,53 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>id_customer</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>start_date</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>monthly_payment</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>cycle</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>